<commit_message>
Sumar hoja Resumen (KPIs) y condición fiscal (IVA recuperable) a la calculadora ML
- Nueva hoja "Resumen": productos cargados, precio/margen/rentabilidad
  promedio, ganancia total, alerta de rentabilidad negativa, producto más
  y menos rentable.
- Parámetro "Condición fiscal del vendedor": si es Responsable Inscripto,
  la Ganancia/Margen/Rentabilidad suman de vuelta el IVA de las comisiones
  ML (crédito fiscal recuperable), en vez de tratarlo siempre como costo
  real. El Ingreso neto recibido sigue reflejando la plata real cobrada.
</commit_message>
<xml_diff>
--- a/recursos/Calculadora-Costos-Rentabilidad-MercadoLibre-Argentina.xlsx
+++ b/recursos/Calculadora-Costos-Rentabilidad-MercadoLibre-Argentina.xlsx
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="Parámetros" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Calculadora" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Notas y Fuentes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Notas y Fuentes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="AlmacenFull" vbProcedure="false">Parámetros!$C$56</definedName>
@@ -18,6 +19,7 @@
     <definedName function="false" hidden="false" name="CatList" vbProcedure="false">Parámetros!$B$6:$B$15</definedName>
     <definedName function="false" hidden="false" name="ComisionClasica" vbProcedure="false">Parámetros!$C$6:$C$15</definedName>
     <definedName function="false" hidden="false" name="ComisionPremium" vbProcedure="false">Parámetros!$D$6:$D$15</definedName>
+    <definedName function="false" hidden="false" name="CondicionFiscal" vbProcedure="false">Parámetros!$C$57</definedName>
     <definedName function="false" hidden="false" name="CostoEnvioPeso" vbProcedure="false">Parámetros!$C$31:$C$35</definedName>
     <definedName function="false" hidden="false" name="CostoFijoTramo" vbProcedure="false">Parámetros!$C$24:$C$26</definedName>
     <definedName function="false" hidden="false" name="CuotasList" vbProcedure="false">Parámetros!$B$47:$B$50</definedName>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="126">
   <si>
     <t xml:space="preserve">PARÁMETROS — Mercado Libre Argentina (editable)</t>
   </si>
@@ -170,7 +172,13 @@
     <t xml:space="preserve">Costo almacenamiento Full por unidad / mes (estimado)</t>
   </si>
   <si>
-    <t xml:space="preserve">IIBB: es una percepción/anticipo de impuesto (ARCA/rentas provinciales), NO un costo real — se descuenta de tu liquidación pero se recupera como crédito fiscal. Se muestra en la Calculadora solo a modo informativo (columna T) y NO se resta en Margen ni Rentabilidad. Almacenamiento Full: costo diario real depende del tamaño del producto y no es público — este es un promedio mensual estimado, ajustalo con tus liquidaciones.</t>
+    <t xml:space="preserve">Condición fiscal del vendedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monotributo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IIBB: es una percepción/anticipo de impuesto (ARCA/rentas provinciales), NO un costo real — se descuenta de tu liquidación pero se recupera como crédito fiscal. Se muestra en la Calculadora solo a modo informativo (columna T) y NO se resta en Margen ni Rentabilidad. Almacenamiento Full: costo diario real depende del tamaño del producto y no es público — este es un promedio mensual estimado, ajustalo con tus liquidaciones. Condición fiscal: si sos Responsable Inscripto, el IVA que te descuenta Mercado Libre sobre sus comisiones es un crédito fiscal recuperable (no es un costo real) y la planilla lo suma de vuelta en la Ganancia/Rentabilidad; el Ingreso neto recibido sigue mostrando la plata que efectivamente cobrás ese mes. Si sos Monotributista o Exento, ese IVA no se recupera y se trata como costo real. Escribí exactamente "Responsable Inscripto" para activar la recuperación.</t>
   </si>
   <si>
     <t xml:space="preserve">CALCULADORA DE COSTOS, MARGEN Y RENTABILIDAD — MERCADO LIBRE ARGENTINA</t>
@@ -179,7 +187,7 @@
     <t xml:space="preserve">Completá una fila por publicación/venta. Cubre las 4 combinaciones: Full con envío gratis, Mercado Envíos sin Full con envío gratis, envío a cargo del comprador (sin envío gratis), precio por debajo y por encima de los $33.000 (umbral de envío gratis obligatorio). Los valores de tarifas se editan en la hoja "Parámetros".</t>
   </si>
   <si>
-    <t xml:space="preserve">Filas 6-9 (fondo naranja) = 4 ejemplos resueltos, no las borres. Filas 10 en adelante = tus productos. Azul = dato que completás vos · Negro = fórmula, no tocar · Verde/rojo en Margen y Rentabilidad = referencia visual.</t>
+    <t xml:space="preserve">Filas 6-9 (fondo naranja) = 4 ejemplos resueltos, no las borres. Filas 10 en adelante = tus productos. Azul = dato que completás vos · Negro = fórmula, no tocar · Verde/rojo en Margen y Rentabilidad = referencia visual. La Ganancia usa la "Condición fiscal" de Parámetros: si sos Responsable Inscripto, el IVA de las comisiones ML se suma de vuelta (es crédito fiscal recuperable, no costo real).</t>
   </si>
   <si>
     <t xml:space="preserve">SKU / Producto</t>
@@ -281,6 +289,42 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
+    <t xml:space="preserve">RESUMEN — TUS PRODUCTOS EN MERCADO LIBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se calcula solo con las filas de la hoja "Calculadora" que tengan categoría cargada (ejemplos + tus productos). Se actualiza solo al agregar filas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productos cargados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio de venta promedio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ganancia total ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen promedio (s/ precio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentabilidad promedio (s/ costo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productos con rentabilidad negativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRODUCTO MÁS Y MENOS RENTABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Más rentable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menos rentable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si hay productos empatados en rentabilidad, la fórmula muestra el primero que encuentra en la lista.</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOTAS, SUPUESTOS Y FUENTES</t>
   </si>
   <si>
@@ -293,6 +337,9 @@
     <t xml:space="preserve">• Hoja "Calculadora": una fila por publicación/venta. Filas 6-9 son 4 ejemplos resueltos que cubren los 4 escenarios pedidos: venta Full con envío gratis, venta sin Full con envío gratis, venta con envío a cargo del comprador, y precios por encima/por debajo de $33.000. Desde la fila 10 podés cargar tus propios productos.</t>
   </si>
   <si>
+    <t xml:space="preserve">• Hoja "Resumen": KPIs agregados de todos los productos cargados en la Calculadora — cantidad, precio/margen/rentabilidad promedio, ganancia total, alerta de productos con rentabilidad negativa, y cuál es tu producto más y menos rentable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Margen = Ganancia / Precio de venta. Rentabilidad = Ganancia / (Costo del producto + otros costos directos). Son dos métricas distintas a propósito: el margen te dice qué % del precio te queda, la rentabilidad te dice cuánto ganás en relación a lo que invertiste.</t>
   </si>
   <si>
@@ -311,10 +358,13 @@
     <t xml:space="preserve">4. El costo de almacenamiento Full es un promedio mensual estimado por unidad. El costo real es diario y depende del tamaño/volumen del producto — ajustalo con tu panel de Fulfillment (vendedores.mercadolibre.com.ar).</t>
   </si>
   <si>
-    <t xml:space="preserve">5. La percepción de IIBB (informativo, columna T de la Calculadora) es un anticipo de impuesto, no un costo definitivo: se recupera como crédito fiscal en tu DDJJ de Ingresos Brutos. Por eso no se resta en Margen ni en Rentabilidad. Si sos Monotributista, normalmente no te retienen IIBB ni podés tomar el IVA como crédito — en ese caso poné 0% en Parámetros!C55 y considerá el IVA como costo real ajustando Parámetros!C54 según corresponda a tu condición fiscal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. El cargo de 12 cuotas sin interés (Parámetros, fila 50) es una estimación no confirmada por fuentes públicas — reemplazalo por el valor real que te muestre Mercado Libre al activar cuotas.</t>
+    <t xml:space="preserve">5. La percepción de IIBB (informativo, columna T de la Calculadora) es un anticipo de impuesto, no un costo definitivo: se recupera como crédito fiscal en tu DDJJ de Ingresos Brutos. Por eso no se resta en Margen ni en Rentabilidad. Si sos Monotributista, normalmente no te retienen IIBB — en ese caso poné 0% en Parámetros!C55.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Condición fiscal (Parámetros!C57): el IVA que Mercado Libre descuenta sobre su comisión + costo fijo/envío + cargo por cuotas SÍ sale de tu liquidación (columna Ingreso neto recibido), pero si sos Responsable Inscripto lo recuperás como crédito fiscal en tu propia DDJJ de IVA — por eso la Ganancia, el Margen y la Rentabilidad lo suman de vuelta. Si sos Monotributista o Exento, ese IVA no se recupera y queda como costo real en Ganancia/Margen/Rentabilidad. Escribí exactamente "Responsable Inscripto" en Parámetros!C57 para activar la recuperación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. El cargo de 12 cuotas sin interés (Parámetros, fila 50) es una estimación no confirmada por fuentes públicas — reemplazalo por el valor real que te muestre Mercado Libre al activar cuotas.</t>
   </si>
   <si>
     <t xml:space="preserve">Fuentes consultadas (julio 2026)</t>
@@ -375,7 +425,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
     <numFmt numFmtId="166" formatCode="\$#,##0"/>
@@ -383,8 +433,9 @@
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="0%"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +528,29 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="20"/>
+      <color rgb="FF203864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="20"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -492,7 +566,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -514,7 +588,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFEEF2FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -526,7 +600,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFEEF2FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF2FA"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -579,7 +659,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -636,6 +716,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -688,6 +772,38 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -696,11 +812,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -717,7 +833,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -733,7 +849,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFEEF2FA"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -754,7 +870,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFCE4D6"/>
       <rgbColor rgb="FF2E75B6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -956,7 +1072,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1420,15 +1536,23 @@
         <v>300</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
+      <c r="C57" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="43.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -1447,7 +1571,7 @@
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1490,36 +1614,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14"/>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
-      <c r="X1" s="14"/>
+      <c r="A1" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
+      <c r="S1" s="15"/>
+      <c r="T1" s="15"/>
+      <c r="U1" s="15"/>
+      <c r="V1" s="15"/>
+      <c r="W1" s="15"/>
+      <c r="X1" s="15"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1545,448 +1669,448 @@
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
-      <c r="V3" s="15"/>
-      <c r="W3" s="15"/>
-      <c r="X3" s="15"/>
+    <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
+      <c r="X3" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="A5" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="G5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="H5" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="I5" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="J5" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="K5" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="N5" s="16" t="s">
+      <c r="L5" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="M5" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="N5" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="Q5" s="16" t="s">
+      <c r="O5" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R5" s="16" t="s">
+      <c r="P5" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="S5" s="16" t="s">
+      <c r="Q5" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="T5" s="16" t="s">
+      <c r="R5" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="U5" s="16" t="s">
+      <c r="S5" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="V5" s="16" t="s">
+      <c r="T5" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="W5" s="16" t="s">
+      <c r="U5" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="X5" s="16" t="s">
+      <c r="V5" s="17" t="s">
         <v>69</v>
       </c>
+      <c r="W5" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="X5" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="18" t="s">
+      <c r="A6" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="19" t="n">
+      <c r="C6" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="20" t="n">
         <v>45000</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="20" t="n">
         <v>22000</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="20" t="n">
         <v>500</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="21" t="n">
         <v>1.2</v>
       </c>
-      <c r="H6" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="I6" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="J6" s="18" t="s">
+      <c r="H6" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="L6" s="22" t="n">
         <f aca="false">IF($B6="","",IFERROR(IF($C6="Premium",INDEX(ComisionPremium,MATCH($B6,CatList,0)),INDEX(ComisionClasica,MATCH($B6,CatList,0))),0))</f>
         <v>0.135</v>
       </c>
-      <c r="M6" s="22" t="n">
+      <c r="M6" s="23" t="n">
         <f aca="false">IF($B6="","",$D6*$L6)</f>
         <v>6075</v>
       </c>
-      <c r="N6" s="22" t="n">
+      <c r="N6" s="23" t="n">
         <f aca="false">IF($B6="","",IFERROR(IF($I6="No",0,IF($D6&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D6,TramoPrecioDesde,1))*IF($H6="Full",1-INDEX(DescuentoFull,MATCH($J6,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G6,TramoPesoDesde,1))*IF($H6="Full",1-INDEX(DescuentoFull,MATCH($J6,ReputacionList,0)),1))),0))</f>
         <v>2250</v>
       </c>
-      <c r="O6" s="22" t="n">
+      <c r="O6" s="23" t="n">
         <f aca="false">IF($B6="","",IFERROR($D6*INDEX(CargoCuotas,MATCH($K6,CuotasList,0)),0))</f>
         <v>0</v>
       </c>
-      <c r="P6" s="22" t="n">
+      <c r="P6" s="23" t="n">
         <f aca="false">IF($B6="","",M6+N6+O6)</f>
         <v>8325</v>
       </c>
-      <c r="Q6" s="22" t="n">
+      <c r="Q6" s="23" t="n">
         <f aca="false">IF($B6="","",P6*IVAParam)</f>
         <v>1748.25</v>
       </c>
-      <c r="R6" s="22" t="n">
+      <c r="R6" s="23" t="n">
         <f aca="false">IF($B6="","",IF($H6="Full",AlmacenFull,0))</f>
         <v>300</v>
       </c>
-      <c r="S6" s="22" t="n">
+      <c r="S6" s="23" t="n">
         <f aca="false">IF($B6="","",P6+Q6+R6)</f>
         <v>10373.25</v>
       </c>
-      <c r="T6" s="22" t="n">
+      <c r="T6" s="23" t="n">
         <f aca="false">IF($B6="","",$D6*IIBBParam)</f>
         <v>1575</v>
       </c>
-      <c r="U6" s="22" t="n">
+      <c r="U6" s="23" t="n">
         <f aca="false">IF($B6="","",$D6-$S6)</f>
         <v>34626.75</v>
       </c>
-      <c r="V6" s="22" t="n">
-        <f aca="false">IF($B6="","",$U6-$E6-$F6)</f>
+      <c r="V6" s="23" t="n">
+        <f aca="false">IF($B6="","",$U6-$E6-$F6+IF(CondicionFiscal="Responsable Inscripto",$Q6,0))</f>
         <v>12126.75</v>
       </c>
-      <c r="W6" s="23" t="n">
+      <c r="W6" s="24" t="n">
         <f aca="false">IF($B6="","",IF($D6=0,0,$V6/$D6))</f>
         <v>0.269483333333333</v>
       </c>
-      <c r="X6" s="23" t="n">
+      <c r="X6" s="24" t="n">
         <f aca="false">IF($B6="","",IF(($E6+$F6)=0,0,$V6/($E6+$F6)))</f>
         <v>0.538966666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>300</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H7" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" s="19" t="n">
-        <v>18000</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>9000</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="G7" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="J7" s="18" t="s">
+      <c r="I7" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="21" t="n">
+      <c r="L7" s="22" t="n">
         <f aca="false">IF($B7="","",IFERROR(IF($C7="Premium",INDEX(ComisionPremium,MATCH($B7,CatList,0)),INDEX(ComisionClasica,MATCH($B7,CatList,0))),0))</f>
         <v>0.15</v>
       </c>
-      <c r="M7" s="22" t="n">
+      <c r="M7" s="23" t="n">
         <f aca="false">IF($B7="","",$D7*$L7)</f>
         <v>2700</v>
       </c>
-      <c r="N7" s="22" t="n">
+      <c r="N7" s="23" t="n">
         <f aca="false">IF($B7="","",IFERROR(IF($I7="No",0,IF($D7&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D7,TramoPrecioDesde,1))*IF($H7="Full",1-INDEX(DescuentoFull,MATCH($J7,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G7,TramoPesoDesde,1))*IF($H7="Full",1-INDEX(DescuentoFull,MATCH($J7,ReputacionList,0)),1))),0))</f>
         <v>1350</v>
       </c>
-      <c r="O7" s="22" t="n">
+      <c r="O7" s="23" t="n">
         <f aca="false">IF($B7="","",IFERROR($D7*INDEX(CargoCuotas,MATCH($K7,CuotasList,0)),0))</f>
         <v>1035</v>
       </c>
-      <c r="P7" s="22" t="n">
+      <c r="P7" s="23" t="n">
         <f aca="false">IF($B7="","",M7+N7+O7)</f>
         <v>5085</v>
       </c>
-      <c r="Q7" s="22" t="n">
+      <c r="Q7" s="23" t="n">
         <f aca="false">IF($B7="","",P7*IVAParam)</f>
         <v>1067.85</v>
       </c>
-      <c r="R7" s="22" t="n">
+      <c r="R7" s="23" t="n">
         <f aca="false">IF($B7="","",IF($H7="Full",AlmacenFull,0))</f>
         <v>300</v>
       </c>
-      <c r="S7" s="22" t="n">
+      <c r="S7" s="23" t="n">
         <f aca="false">IF($B7="","",P7+Q7+R7)</f>
         <v>6452.85</v>
       </c>
-      <c r="T7" s="22" t="n">
+      <c r="T7" s="23" t="n">
         <f aca="false">IF($B7="","",$D7*IIBBParam)</f>
         <v>630</v>
       </c>
-      <c r="U7" s="22" t="n">
+      <c r="U7" s="23" t="n">
         <f aca="false">IF($B7="","",$D7-$S7)</f>
         <v>11547.15</v>
       </c>
-      <c r="V7" s="22" t="n">
-        <f aca="false">IF($B7="","",$U7-$E7-$F7)</f>
+      <c r="V7" s="23" t="n">
+        <f aca="false">IF($B7="","",$U7-$E7-$F7+IF(CondicionFiscal="Responsable Inscripto",$Q7,0))</f>
         <v>2247.15</v>
       </c>
-      <c r="W7" s="23" t="n">
+      <c r="W7" s="24" t="n">
         <f aca="false">IF($B7="","",IF($D7=0,0,$V7/$D7))</f>
         <v>0.124841666666667</v>
       </c>
-      <c r="X7" s="23" t="n">
+      <c r="X7" s="24" t="n">
         <f aca="false">IF($B7="","",IF(($E7+$F7)=0,0,$V7/($E7+$F7)))</f>
         <v>0.241629032258064</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" s="19" t="n">
-        <v>12000</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18" t="n">
+      <c r="J8" s="19"/>
+      <c r="K8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="21" t="n">
+      <c r="L8" s="22" t="n">
         <f aca="false">IF($B8="","",IFERROR(IF($C8="Premium",INDEX(ComisionPremium,MATCH($B8,CatList,0)),INDEX(ComisionClasica,MATCH($B8,CatList,0))),0))</f>
         <v>0.13</v>
       </c>
-      <c r="M8" s="22" t="n">
+      <c r="M8" s="23" t="n">
         <f aca="false">IF($B8="","",$D8*$L8)</f>
         <v>1560</v>
       </c>
-      <c r="N8" s="22" t="n">
+      <c r="N8" s="23" t="n">
         <f aca="false">IF($B8="","",IFERROR(IF($I8="No",0,IF($D8&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D8,TramoPrecioDesde,1))*IF($H8="Full",1-INDEX(DescuentoFull,MATCH($J8,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G8,TramoPesoDesde,1))*IF($H8="Full",1-INDEX(DescuentoFull,MATCH($J8,ReputacionList,0)),1))),0))</f>
         <v>1100</v>
       </c>
-      <c r="O8" s="22" t="n">
+      <c r="O8" s="23" t="n">
         <f aca="false">IF($B8="","",IFERROR($D8*INDEX(CargoCuotas,MATCH($K8,CuotasList,0)),0))</f>
         <v>0</v>
       </c>
-      <c r="P8" s="22" t="n">
+      <c r="P8" s="23" t="n">
         <f aca="false">IF($B8="","",M8+N8+O8)</f>
         <v>2660</v>
       </c>
-      <c r="Q8" s="22" t="n">
+      <c r="Q8" s="23" t="n">
         <f aca="false">IF($B8="","",P8*IVAParam)</f>
         <v>558.6</v>
       </c>
-      <c r="R8" s="22" t="n">
+      <c r="R8" s="23" t="n">
         <f aca="false">IF($B8="","",IF($H8="Full",AlmacenFull,0))</f>
         <v>0</v>
       </c>
-      <c r="S8" s="22" t="n">
+      <c r="S8" s="23" t="n">
         <f aca="false">IF($B8="","",P8+Q8+R8)</f>
         <v>3218.6</v>
       </c>
-      <c r="T8" s="22" t="n">
+      <c r="T8" s="23" t="n">
         <f aca="false">IF($B8="","",$D8*IIBBParam)</f>
         <v>420</v>
       </c>
-      <c r="U8" s="22" t="n">
+      <c r="U8" s="23" t="n">
         <f aca="false">IF($B8="","",$D8-$S8)</f>
         <v>8781.4</v>
       </c>
-      <c r="V8" s="22" t="n">
-        <f aca="false">IF($B8="","",$U8-$E8-$F8)</f>
+      <c r="V8" s="23" t="n">
+        <f aca="false">IF($B8="","",$U8-$E8-$F8+IF(CondicionFiscal="Responsable Inscripto",$Q8,0))</f>
         <v>2581.4</v>
       </c>
-      <c r="W8" s="23" t="n">
+      <c r="W8" s="24" t="n">
         <f aca="false">IF($B8="","",IF($D8=0,0,$V8/$D8))</f>
         <v>0.215116666666667</v>
       </c>
-      <c r="X8" s="23" t="n">
+      <c r="X8" s="24" t="n">
         <f aca="false">IF($B8="","",IF(($E8+$F8)=0,0,$V8/($E8+$F8)))</f>
         <v>0.416354838709677</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="18" t="s">
+      <c r="A9" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="19" t="n">
+      <c r="C9" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="20" t="n">
         <v>8000</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="20" t="n">
         <v>4000</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="H9" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="I9" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18" t="n">
+      <c r="H9" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="21" t="n">
+      <c r="L9" s="22" t="n">
         <f aca="false">IF($B9="","",IFERROR(IF($C9="Premium",INDEX(ComisionPremium,MATCH($B9,CatList,0)),INDEX(ComisionClasica,MATCH($B9,CatList,0))),0))</f>
         <v>0.135</v>
       </c>
-      <c r="M9" s="22" t="n">
+      <c r="M9" s="23" t="n">
         <f aca="false">IF($B9="","",$D9*$L9)</f>
         <v>1080</v>
       </c>
-      <c r="N9" s="22" t="n">
+      <c r="N9" s="23" t="n">
         <f aca="false">IF($B9="","",IFERROR(IF($I9="No",0,IF($D9&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D9,TramoPrecioDesde,1))*IF($H9="Full",1-INDEX(DescuentoFull,MATCH($J9,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G9,TramoPesoDesde,1))*IF($H9="Full",1-INDEX(DescuentoFull,MATCH($J9,ReputacionList,0)),1))),0))</f>
         <v>0</v>
       </c>
-      <c r="O9" s="22" t="n">
+      <c r="O9" s="23" t="n">
         <f aca="false">IF($B9="","",IFERROR($D9*INDEX(CargoCuotas,MATCH($K9,CuotasList,0)),0))</f>
         <v>0</v>
       </c>
-      <c r="P9" s="22" t="n">
+      <c r="P9" s="23" t="n">
         <f aca="false">IF($B9="","",M9+N9+O9)</f>
         <v>1080</v>
       </c>
-      <c r="Q9" s="22" t="n">
+      <c r="Q9" s="23" t="n">
         <f aca="false">IF($B9="","",P9*IVAParam)</f>
         <v>226.8</v>
       </c>
-      <c r="R9" s="22" t="n">
+      <c r="R9" s="23" t="n">
         <f aca="false">IF($B9="","",IF($H9="Full",AlmacenFull,0))</f>
         <v>0</v>
       </c>
-      <c r="S9" s="22" t="n">
+      <c r="S9" s="23" t="n">
         <f aca="false">IF($B9="","",P9+Q9+R9)</f>
         <v>1306.8</v>
       </c>
-      <c r="T9" s="22" t="n">
+      <c r="T9" s="23" t="n">
         <f aca="false">IF($B9="","",$D9*IIBBParam)</f>
         <v>280</v>
       </c>
-      <c r="U9" s="22" t="n">
+      <c r="U9" s="23" t="n">
         <f aca="false">IF($B9="","",$D9-$S9)</f>
         <v>6693.2</v>
       </c>
-      <c r="V9" s="22" t="n">
-        <f aca="false">IF($B9="","",$U9-$E9-$F9)</f>
+      <c r="V9" s="23" t="n">
+        <f aca="false">IF($B9="","",$U9-$E9-$F9+IF(CondicionFiscal="Responsable Inscripto",$Q9,0))</f>
         <v>2593.2</v>
       </c>
-      <c r="W9" s="23" t="n">
+      <c r="W9" s="24" t="n">
         <f aca="false">IF($B9="","",IF($D9=0,0,$V9/$D9))</f>
         <v>0.32415</v>
       </c>
-      <c r="X9" s="23" t="n">
+      <c r="X9" s="24" t="n">
         <f aca="false">IF($B9="","",IF(($E9+$F9)=0,0,$V9/($E9+$F9)))</f>
         <v>0.632487804878049</v>
       </c>
@@ -2003,55 +2127,55 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
-      <c r="L10" s="24" t="str">
+      <c r="L10" s="25" t="str">
         <f aca="false">IF($B10="","",IFERROR(IF($C10="Premium",INDEX(ComisionPremium,MATCH($B10,CatList,0)),INDEX(ComisionClasica,MATCH($B10,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M10" s="25" t="str">
+      <c r="M10" s="26" t="str">
         <f aca="false">IF($B10="","",$D10*$L10)</f>
         <v/>
       </c>
-      <c r="N10" s="25" t="str">
+      <c r="N10" s="26" t="str">
         <f aca="false">IF($B10="","",IFERROR(IF($I10="No",0,IF($D10&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D10,TramoPrecioDesde,1))*IF($H10="Full",1-INDEX(DescuentoFull,MATCH($J10,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G10,TramoPesoDesde,1))*IF($H10="Full",1-INDEX(DescuentoFull,MATCH($J10,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O10" s="25" t="str">
+      <c r="O10" s="26" t="str">
         <f aca="false">IF($B10="","",IFERROR($D10*INDEX(CargoCuotas,MATCH($K10,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P10" s="25" t="str">
+      <c r="P10" s="26" t="str">
         <f aca="false">IF($B10="","",M10+N10+O10)</f>
         <v/>
       </c>
-      <c r="Q10" s="25" t="str">
+      <c r="Q10" s="26" t="str">
         <f aca="false">IF($B10="","",P10*IVAParam)</f>
         <v/>
       </c>
-      <c r="R10" s="25" t="str">
+      <c r="R10" s="26" t="str">
         <f aca="false">IF($B10="","",IF($H10="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S10" s="25" t="str">
+      <c r="S10" s="26" t="str">
         <f aca="false">IF($B10="","",P10+Q10+R10)</f>
         <v/>
       </c>
-      <c r="T10" s="25" t="str">
+      <c r="T10" s="26" t="str">
         <f aca="false">IF($B10="","",$D10*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U10" s="25" t="str">
+      <c r="U10" s="26" t="str">
         <f aca="false">IF($B10="","",$D10-$S10)</f>
         <v/>
       </c>
-      <c r="V10" s="25" t="str">
-        <f aca="false">IF($B10="","",$U10-$E10-$F10)</f>
-        <v/>
-      </c>
-      <c r="W10" s="26" t="str">
+      <c r="V10" s="26" t="str">
+        <f aca="false">IF($B10="","",$U10-$E10-$F10+IF(CondicionFiscal="Responsable Inscripto",$Q10,0))</f>
+        <v/>
+      </c>
+      <c r="W10" s="27" t="str">
         <f aca="false">IF($B10="","",IF($D10=0,0,$V10/$D10))</f>
         <v/>
       </c>
-      <c r="X10" s="26" t="str">
+      <c r="X10" s="27" t="str">
         <f aca="false">IF($B10="","",IF(($E10+$F10)=0,0,$V10/($E10+$F10)))</f>
         <v/>
       </c>
@@ -2068,55 +2192,55 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="L11" s="24" t="str">
+      <c r="L11" s="25" t="str">
         <f aca="false">IF($B11="","",IFERROR(IF($C11="Premium",INDEX(ComisionPremium,MATCH($B11,CatList,0)),INDEX(ComisionClasica,MATCH($B11,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M11" s="25" t="str">
+      <c r="M11" s="26" t="str">
         <f aca="false">IF($B11="","",$D11*$L11)</f>
         <v/>
       </c>
-      <c r="N11" s="25" t="str">
+      <c r="N11" s="26" t="str">
         <f aca="false">IF($B11="","",IFERROR(IF($I11="No",0,IF($D11&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D11,TramoPrecioDesde,1))*IF($H11="Full",1-INDEX(DescuentoFull,MATCH($J11,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G11,TramoPesoDesde,1))*IF($H11="Full",1-INDEX(DescuentoFull,MATCH($J11,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O11" s="25" t="str">
+      <c r="O11" s="26" t="str">
         <f aca="false">IF($B11="","",IFERROR($D11*INDEX(CargoCuotas,MATCH($K11,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P11" s="25" t="str">
+      <c r="P11" s="26" t="str">
         <f aca="false">IF($B11="","",M11+N11+O11)</f>
         <v/>
       </c>
-      <c r="Q11" s="25" t="str">
+      <c r="Q11" s="26" t="str">
         <f aca="false">IF($B11="","",P11*IVAParam)</f>
         <v/>
       </c>
-      <c r="R11" s="25" t="str">
+      <c r="R11" s="26" t="str">
         <f aca="false">IF($B11="","",IF($H11="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S11" s="25" t="str">
+      <c r="S11" s="26" t="str">
         <f aca="false">IF($B11="","",P11+Q11+R11)</f>
         <v/>
       </c>
-      <c r="T11" s="25" t="str">
+      <c r="T11" s="26" t="str">
         <f aca="false">IF($B11="","",$D11*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U11" s="25" t="str">
+      <c r="U11" s="26" t="str">
         <f aca="false">IF($B11="","",$D11-$S11)</f>
         <v/>
       </c>
-      <c r="V11" s="25" t="str">
-        <f aca="false">IF($B11="","",$U11-$E11-$F11)</f>
-        <v/>
-      </c>
-      <c r="W11" s="26" t="str">
+      <c r="V11" s="26" t="str">
+        <f aca="false">IF($B11="","",$U11-$E11-$F11+IF(CondicionFiscal="Responsable Inscripto",$Q11,0))</f>
+        <v/>
+      </c>
+      <c r="W11" s="27" t="str">
         <f aca="false">IF($B11="","",IF($D11=0,0,$V11/$D11))</f>
         <v/>
       </c>
-      <c r="X11" s="26" t="str">
+      <c r="X11" s="27" t="str">
         <f aca="false">IF($B11="","",IF(($E11+$F11)=0,0,$V11/($E11+$F11)))</f>
         <v/>
       </c>
@@ -2133,55 +2257,55 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="L12" s="24" t="str">
+      <c r="L12" s="25" t="str">
         <f aca="false">IF($B12="","",IFERROR(IF($C12="Premium",INDEX(ComisionPremium,MATCH($B12,CatList,0)),INDEX(ComisionClasica,MATCH($B12,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M12" s="25" t="str">
+      <c r="M12" s="26" t="str">
         <f aca="false">IF($B12="","",$D12*$L12)</f>
         <v/>
       </c>
-      <c r="N12" s="25" t="str">
+      <c r="N12" s="26" t="str">
         <f aca="false">IF($B12="","",IFERROR(IF($I12="No",0,IF($D12&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D12,TramoPrecioDesde,1))*IF($H12="Full",1-INDEX(DescuentoFull,MATCH($J12,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G12,TramoPesoDesde,1))*IF($H12="Full",1-INDEX(DescuentoFull,MATCH($J12,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O12" s="25" t="str">
+      <c r="O12" s="26" t="str">
         <f aca="false">IF($B12="","",IFERROR($D12*INDEX(CargoCuotas,MATCH($K12,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P12" s="25" t="str">
+      <c r="P12" s="26" t="str">
         <f aca="false">IF($B12="","",M12+N12+O12)</f>
         <v/>
       </c>
-      <c r="Q12" s="25" t="str">
+      <c r="Q12" s="26" t="str">
         <f aca="false">IF($B12="","",P12*IVAParam)</f>
         <v/>
       </c>
-      <c r="R12" s="25" t="str">
+      <c r="R12" s="26" t="str">
         <f aca="false">IF($B12="","",IF($H12="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S12" s="25" t="str">
+      <c r="S12" s="26" t="str">
         <f aca="false">IF($B12="","",P12+Q12+R12)</f>
         <v/>
       </c>
-      <c r="T12" s="25" t="str">
+      <c r="T12" s="26" t="str">
         <f aca="false">IF($B12="","",$D12*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U12" s="25" t="str">
+      <c r="U12" s="26" t="str">
         <f aca="false">IF($B12="","",$D12-$S12)</f>
         <v/>
       </c>
-      <c r="V12" s="25" t="str">
-        <f aca="false">IF($B12="","",$U12-$E12-$F12)</f>
-        <v/>
-      </c>
-      <c r="W12" s="26" t="str">
+      <c r="V12" s="26" t="str">
+        <f aca="false">IF($B12="","",$U12-$E12-$F12+IF(CondicionFiscal="Responsable Inscripto",$Q12,0))</f>
+        <v/>
+      </c>
+      <c r="W12" s="27" t="str">
         <f aca="false">IF($B12="","",IF($D12=0,0,$V12/$D12))</f>
         <v/>
       </c>
-      <c r="X12" s="26" t="str">
+      <c r="X12" s="27" t="str">
         <f aca="false">IF($B12="","",IF(($E12+$F12)=0,0,$V12/($E12+$F12)))</f>
         <v/>
       </c>
@@ -2198,55 +2322,55 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
-      <c r="L13" s="24" t="str">
+      <c r="L13" s="25" t="str">
         <f aca="false">IF($B13="","",IFERROR(IF($C13="Premium",INDEX(ComisionPremium,MATCH($B13,CatList,0)),INDEX(ComisionClasica,MATCH($B13,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M13" s="25" t="str">
+      <c r="M13" s="26" t="str">
         <f aca="false">IF($B13="","",$D13*$L13)</f>
         <v/>
       </c>
-      <c r="N13" s="25" t="str">
+      <c r="N13" s="26" t="str">
         <f aca="false">IF($B13="","",IFERROR(IF($I13="No",0,IF($D13&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D13,TramoPrecioDesde,1))*IF($H13="Full",1-INDEX(DescuentoFull,MATCH($J13,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G13,TramoPesoDesde,1))*IF($H13="Full",1-INDEX(DescuentoFull,MATCH($J13,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O13" s="25" t="str">
+      <c r="O13" s="26" t="str">
         <f aca="false">IF($B13="","",IFERROR($D13*INDEX(CargoCuotas,MATCH($K13,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P13" s="25" t="str">
+      <c r="P13" s="26" t="str">
         <f aca="false">IF($B13="","",M13+N13+O13)</f>
         <v/>
       </c>
-      <c r="Q13" s="25" t="str">
+      <c r="Q13" s="26" t="str">
         <f aca="false">IF($B13="","",P13*IVAParam)</f>
         <v/>
       </c>
-      <c r="R13" s="25" t="str">
+      <c r="R13" s="26" t="str">
         <f aca="false">IF($B13="","",IF($H13="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S13" s="25" t="str">
+      <c r="S13" s="26" t="str">
         <f aca="false">IF($B13="","",P13+Q13+R13)</f>
         <v/>
       </c>
-      <c r="T13" s="25" t="str">
+      <c r="T13" s="26" t="str">
         <f aca="false">IF($B13="","",$D13*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U13" s="25" t="str">
+      <c r="U13" s="26" t="str">
         <f aca="false">IF($B13="","",$D13-$S13)</f>
         <v/>
       </c>
-      <c r="V13" s="25" t="str">
-        <f aca="false">IF($B13="","",$U13-$E13-$F13)</f>
-        <v/>
-      </c>
-      <c r="W13" s="26" t="str">
+      <c r="V13" s="26" t="str">
+        <f aca="false">IF($B13="","",$U13-$E13-$F13+IF(CondicionFiscal="Responsable Inscripto",$Q13,0))</f>
+        <v/>
+      </c>
+      <c r="W13" s="27" t="str">
         <f aca="false">IF($B13="","",IF($D13=0,0,$V13/$D13))</f>
         <v/>
       </c>
-      <c r="X13" s="26" t="str">
+      <c r="X13" s="27" t="str">
         <f aca="false">IF($B13="","",IF(($E13+$F13)=0,0,$V13/($E13+$F13)))</f>
         <v/>
       </c>
@@ -2263,55 +2387,55 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
-      <c r="L14" s="24" t="str">
+      <c r="L14" s="25" t="str">
         <f aca="false">IF($B14="","",IFERROR(IF($C14="Premium",INDEX(ComisionPremium,MATCH($B14,CatList,0)),INDEX(ComisionClasica,MATCH($B14,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M14" s="25" t="str">
+      <c r="M14" s="26" t="str">
         <f aca="false">IF($B14="","",$D14*$L14)</f>
         <v/>
       </c>
-      <c r="N14" s="25" t="str">
+      <c r="N14" s="26" t="str">
         <f aca="false">IF($B14="","",IFERROR(IF($I14="No",0,IF($D14&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D14,TramoPrecioDesde,1))*IF($H14="Full",1-INDEX(DescuentoFull,MATCH($J14,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G14,TramoPesoDesde,1))*IF($H14="Full",1-INDEX(DescuentoFull,MATCH($J14,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O14" s="25" t="str">
+      <c r="O14" s="26" t="str">
         <f aca="false">IF($B14="","",IFERROR($D14*INDEX(CargoCuotas,MATCH($K14,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P14" s="25" t="str">
+      <c r="P14" s="26" t="str">
         <f aca="false">IF($B14="","",M14+N14+O14)</f>
         <v/>
       </c>
-      <c r="Q14" s="25" t="str">
+      <c r="Q14" s="26" t="str">
         <f aca="false">IF($B14="","",P14*IVAParam)</f>
         <v/>
       </c>
-      <c r="R14" s="25" t="str">
+      <c r="R14" s="26" t="str">
         <f aca="false">IF($B14="","",IF($H14="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S14" s="25" t="str">
+      <c r="S14" s="26" t="str">
         <f aca="false">IF($B14="","",P14+Q14+R14)</f>
         <v/>
       </c>
-      <c r="T14" s="25" t="str">
+      <c r="T14" s="26" t="str">
         <f aca="false">IF($B14="","",$D14*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U14" s="25" t="str">
+      <c r="U14" s="26" t="str">
         <f aca="false">IF($B14="","",$D14-$S14)</f>
         <v/>
       </c>
-      <c r="V14" s="25" t="str">
-        <f aca="false">IF($B14="","",$U14-$E14-$F14)</f>
-        <v/>
-      </c>
-      <c r="W14" s="26" t="str">
+      <c r="V14" s="26" t="str">
+        <f aca="false">IF($B14="","",$U14-$E14-$F14+IF(CondicionFiscal="Responsable Inscripto",$Q14,0))</f>
+        <v/>
+      </c>
+      <c r="W14" s="27" t="str">
         <f aca="false">IF($B14="","",IF($D14=0,0,$V14/$D14))</f>
         <v/>
       </c>
-      <c r="X14" s="26" t="str">
+      <c r="X14" s="27" t="str">
         <f aca="false">IF($B14="","",IF(($E14+$F14)=0,0,$V14/($E14+$F14)))</f>
         <v/>
       </c>
@@ -2328,55 +2452,55 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
-      <c r="L15" s="24" t="str">
+      <c r="L15" s="25" t="str">
         <f aca="false">IF($B15="","",IFERROR(IF($C15="Premium",INDEX(ComisionPremium,MATCH($B15,CatList,0)),INDEX(ComisionClasica,MATCH($B15,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M15" s="25" t="str">
+      <c r="M15" s="26" t="str">
         <f aca="false">IF($B15="","",$D15*$L15)</f>
         <v/>
       </c>
-      <c r="N15" s="25" t="str">
+      <c r="N15" s="26" t="str">
         <f aca="false">IF($B15="","",IFERROR(IF($I15="No",0,IF($D15&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D15,TramoPrecioDesde,1))*IF($H15="Full",1-INDEX(DescuentoFull,MATCH($J15,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G15,TramoPesoDesde,1))*IF($H15="Full",1-INDEX(DescuentoFull,MATCH($J15,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O15" s="25" t="str">
+      <c r="O15" s="26" t="str">
         <f aca="false">IF($B15="","",IFERROR($D15*INDEX(CargoCuotas,MATCH($K15,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P15" s="25" t="str">
+      <c r="P15" s="26" t="str">
         <f aca="false">IF($B15="","",M15+N15+O15)</f>
         <v/>
       </c>
-      <c r="Q15" s="25" t="str">
+      <c r="Q15" s="26" t="str">
         <f aca="false">IF($B15="","",P15*IVAParam)</f>
         <v/>
       </c>
-      <c r="R15" s="25" t="str">
+      <c r="R15" s="26" t="str">
         <f aca="false">IF($B15="","",IF($H15="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S15" s="25" t="str">
+      <c r="S15" s="26" t="str">
         <f aca="false">IF($B15="","",P15+Q15+R15)</f>
         <v/>
       </c>
-      <c r="T15" s="25" t="str">
+      <c r="T15" s="26" t="str">
         <f aca="false">IF($B15="","",$D15*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U15" s="25" t="str">
+      <c r="U15" s="26" t="str">
         <f aca="false">IF($B15="","",$D15-$S15)</f>
         <v/>
       </c>
-      <c r="V15" s="25" t="str">
-        <f aca="false">IF($B15="","",$U15-$E15-$F15)</f>
-        <v/>
-      </c>
-      <c r="W15" s="26" t="str">
+      <c r="V15" s="26" t="str">
+        <f aca="false">IF($B15="","",$U15-$E15-$F15+IF(CondicionFiscal="Responsable Inscripto",$Q15,0))</f>
+        <v/>
+      </c>
+      <c r="W15" s="27" t="str">
         <f aca="false">IF($B15="","",IF($D15=0,0,$V15/$D15))</f>
         <v/>
       </c>
-      <c r="X15" s="26" t="str">
+      <c r="X15" s="27" t="str">
         <f aca="false">IF($B15="","",IF(($E15+$F15)=0,0,$V15/($E15+$F15)))</f>
         <v/>
       </c>
@@ -2393,55 +2517,55 @@
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
-      <c r="L16" s="24" t="str">
+      <c r="L16" s="25" t="str">
         <f aca="false">IF($B16="","",IFERROR(IF($C16="Premium",INDEX(ComisionPremium,MATCH($B16,CatList,0)),INDEX(ComisionClasica,MATCH($B16,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M16" s="25" t="str">
+      <c r="M16" s="26" t="str">
         <f aca="false">IF($B16="","",$D16*$L16)</f>
         <v/>
       </c>
-      <c r="N16" s="25" t="str">
+      <c r="N16" s="26" t="str">
         <f aca="false">IF($B16="","",IFERROR(IF($I16="No",0,IF($D16&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D16,TramoPrecioDesde,1))*IF($H16="Full",1-INDEX(DescuentoFull,MATCH($J16,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G16,TramoPesoDesde,1))*IF($H16="Full",1-INDEX(DescuentoFull,MATCH($J16,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O16" s="25" t="str">
+      <c r="O16" s="26" t="str">
         <f aca="false">IF($B16="","",IFERROR($D16*INDEX(CargoCuotas,MATCH($K16,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P16" s="25" t="str">
+      <c r="P16" s="26" t="str">
         <f aca="false">IF($B16="","",M16+N16+O16)</f>
         <v/>
       </c>
-      <c r="Q16" s="25" t="str">
+      <c r="Q16" s="26" t="str">
         <f aca="false">IF($B16="","",P16*IVAParam)</f>
         <v/>
       </c>
-      <c r="R16" s="25" t="str">
+      <c r="R16" s="26" t="str">
         <f aca="false">IF($B16="","",IF($H16="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S16" s="25" t="str">
+      <c r="S16" s="26" t="str">
         <f aca="false">IF($B16="","",P16+Q16+R16)</f>
         <v/>
       </c>
-      <c r="T16" s="25" t="str">
+      <c r="T16" s="26" t="str">
         <f aca="false">IF($B16="","",$D16*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U16" s="25" t="str">
+      <c r="U16" s="26" t="str">
         <f aca="false">IF($B16="","",$D16-$S16)</f>
         <v/>
       </c>
-      <c r="V16" s="25" t="str">
-        <f aca="false">IF($B16="","",$U16-$E16-$F16)</f>
-        <v/>
-      </c>
-      <c r="W16" s="26" t="str">
+      <c r="V16" s="26" t="str">
+        <f aca="false">IF($B16="","",$U16-$E16-$F16+IF(CondicionFiscal="Responsable Inscripto",$Q16,0))</f>
+        <v/>
+      </c>
+      <c r="W16" s="27" t="str">
         <f aca="false">IF($B16="","",IF($D16=0,0,$V16/$D16))</f>
         <v/>
       </c>
-      <c r="X16" s="26" t="str">
+      <c r="X16" s="27" t="str">
         <f aca="false">IF($B16="","",IF(($E16+$F16)=0,0,$V16/($E16+$F16)))</f>
         <v/>
       </c>
@@ -2458,55 +2582,55 @@
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
-      <c r="L17" s="24" t="str">
+      <c r="L17" s="25" t="str">
         <f aca="false">IF($B17="","",IFERROR(IF($C17="Premium",INDEX(ComisionPremium,MATCH($B17,CatList,0)),INDEX(ComisionClasica,MATCH($B17,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M17" s="25" t="str">
+      <c r="M17" s="26" t="str">
         <f aca="false">IF($B17="","",$D17*$L17)</f>
         <v/>
       </c>
-      <c r="N17" s="25" t="str">
+      <c r="N17" s="26" t="str">
         <f aca="false">IF($B17="","",IFERROR(IF($I17="No",0,IF($D17&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D17,TramoPrecioDesde,1))*IF($H17="Full",1-INDEX(DescuentoFull,MATCH($J17,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G17,TramoPesoDesde,1))*IF($H17="Full",1-INDEX(DescuentoFull,MATCH($J17,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O17" s="25" t="str">
+      <c r="O17" s="26" t="str">
         <f aca="false">IF($B17="","",IFERROR($D17*INDEX(CargoCuotas,MATCH($K17,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P17" s="25" t="str">
+      <c r="P17" s="26" t="str">
         <f aca="false">IF($B17="","",M17+N17+O17)</f>
         <v/>
       </c>
-      <c r="Q17" s="25" t="str">
+      <c r="Q17" s="26" t="str">
         <f aca="false">IF($B17="","",P17*IVAParam)</f>
         <v/>
       </c>
-      <c r="R17" s="25" t="str">
+      <c r="R17" s="26" t="str">
         <f aca="false">IF($B17="","",IF($H17="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S17" s="25" t="str">
+      <c r="S17" s="26" t="str">
         <f aca="false">IF($B17="","",P17+Q17+R17)</f>
         <v/>
       </c>
-      <c r="T17" s="25" t="str">
+      <c r="T17" s="26" t="str">
         <f aca="false">IF($B17="","",$D17*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U17" s="25" t="str">
+      <c r="U17" s="26" t="str">
         <f aca="false">IF($B17="","",$D17-$S17)</f>
         <v/>
       </c>
-      <c r="V17" s="25" t="str">
-        <f aca="false">IF($B17="","",$U17-$E17-$F17)</f>
-        <v/>
-      </c>
-      <c r="W17" s="26" t="str">
+      <c r="V17" s="26" t="str">
+        <f aca="false">IF($B17="","",$U17-$E17-$F17+IF(CondicionFiscal="Responsable Inscripto",$Q17,0))</f>
+        <v/>
+      </c>
+      <c r="W17" s="27" t="str">
         <f aca="false">IF($B17="","",IF($D17=0,0,$V17/$D17))</f>
         <v/>
       </c>
-      <c r="X17" s="26" t="str">
+      <c r="X17" s="27" t="str">
         <f aca="false">IF($B17="","",IF(($E17+$F17)=0,0,$V17/($E17+$F17)))</f>
         <v/>
       </c>
@@ -2523,55 +2647,55 @@
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
-      <c r="L18" s="24" t="str">
+      <c r="L18" s="25" t="str">
         <f aca="false">IF($B18="","",IFERROR(IF($C18="Premium",INDEX(ComisionPremium,MATCH($B18,CatList,0)),INDEX(ComisionClasica,MATCH($B18,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M18" s="25" t="str">
+      <c r="M18" s="26" t="str">
         <f aca="false">IF($B18="","",$D18*$L18)</f>
         <v/>
       </c>
-      <c r="N18" s="25" t="str">
+      <c r="N18" s="26" t="str">
         <f aca="false">IF($B18="","",IFERROR(IF($I18="No",0,IF($D18&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D18,TramoPrecioDesde,1))*IF($H18="Full",1-INDEX(DescuentoFull,MATCH($J18,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G18,TramoPesoDesde,1))*IF($H18="Full",1-INDEX(DescuentoFull,MATCH($J18,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O18" s="25" t="str">
+      <c r="O18" s="26" t="str">
         <f aca="false">IF($B18="","",IFERROR($D18*INDEX(CargoCuotas,MATCH($K18,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P18" s="25" t="str">
+      <c r="P18" s="26" t="str">
         <f aca="false">IF($B18="","",M18+N18+O18)</f>
         <v/>
       </c>
-      <c r="Q18" s="25" t="str">
+      <c r="Q18" s="26" t="str">
         <f aca="false">IF($B18="","",P18*IVAParam)</f>
         <v/>
       </c>
-      <c r="R18" s="25" t="str">
+      <c r="R18" s="26" t="str">
         <f aca="false">IF($B18="","",IF($H18="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S18" s="25" t="str">
+      <c r="S18" s="26" t="str">
         <f aca="false">IF($B18="","",P18+Q18+R18)</f>
         <v/>
       </c>
-      <c r="T18" s="25" t="str">
+      <c r="T18" s="26" t="str">
         <f aca="false">IF($B18="","",$D18*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U18" s="25" t="str">
+      <c r="U18" s="26" t="str">
         <f aca="false">IF($B18="","",$D18-$S18)</f>
         <v/>
       </c>
-      <c r="V18" s="25" t="str">
-        <f aca="false">IF($B18="","",$U18-$E18-$F18)</f>
-        <v/>
-      </c>
-      <c r="W18" s="26" t="str">
+      <c r="V18" s="26" t="str">
+        <f aca="false">IF($B18="","",$U18-$E18-$F18+IF(CondicionFiscal="Responsable Inscripto",$Q18,0))</f>
+        <v/>
+      </c>
+      <c r="W18" s="27" t="str">
         <f aca="false">IF($B18="","",IF($D18=0,0,$V18/$D18))</f>
         <v/>
       </c>
-      <c r="X18" s="26" t="str">
+      <c r="X18" s="27" t="str">
         <f aca="false">IF($B18="","",IF(($E18+$F18)=0,0,$V18/($E18+$F18)))</f>
         <v/>
       </c>
@@ -2588,55 +2712,55 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
-      <c r="L19" s="24" t="str">
+      <c r="L19" s="25" t="str">
         <f aca="false">IF($B19="","",IFERROR(IF($C19="Premium",INDEX(ComisionPremium,MATCH($B19,CatList,0)),INDEX(ComisionClasica,MATCH($B19,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M19" s="25" t="str">
+      <c r="M19" s="26" t="str">
         <f aca="false">IF($B19="","",$D19*$L19)</f>
         <v/>
       </c>
-      <c r="N19" s="25" t="str">
+      <c r="N19" s="26" t="str">
         <f aca="false">IF($B19="","",IFERROR(IF($I19="No",0,IF($D19&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D19,TramoPrecioDesde,1))*IF($H19="Full",1-INDEX(DescuentoFull,MATCH($J19,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G19,TramoPesoDesde,1))*IF($H19="Full",1-INDEX(DescuentoFull,MATCH($J19,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O19" s="25" t="str">
+      <c r="O19" s="26" t="str">
         <f aca="false">IF($B19="","",IFERROR($D19*INDEX(CargoCuotas,MATCH($K19,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P19" s="25" t="str">
+      <c r="P19" s="26" t="str">
         <f aca="false">IF($B19="","",M19+N19+O19)</f>
         <v/>
       </c>
-      <c r="Q19" s="25" t="str">
+      <c r="Q19" s="26" t="str">
         <f aca="false">IF($B19="","",P19*IVAParam)</f>
         <v/>
       </c>
-      <c r="R19" s="25" t="str">
+      <c r="R19" s="26" t="str">
         <f aca="false">IF($B19="","",IF($H19="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S19" s="25" t="str">
+      <c r="S19" s="26" t="str">
         <f aca="false">IF($B19="","",P19+Q19+R19)</f>
         <v/>
       </c>
-      <c r="T19" s="25" t="str">
+      <c r="T19" s="26" t="str">
         <f aca="false">IF($B19="","",$D19*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U19" s="25" t="str">
+      <c r="U19" s="26" t="str">
         <f aca="false">IF($B19="","",$D19-$S19)</f>
         <v/>
       </c>
-      <c r="V19" s="25" t="str">
-        <f aca="false">IF($B19="","",$U19-$E19-$F19)</f>
-        <v/>
-      </c>
-      <c r="W19" s="26" t="str">
+      <c r="V19" s="26" t="str">
+        <f aca="false">IF($B19="","",$U19-$E19-$F19+IF(CondicionFiscal="Responsable Inscripto",$Q19,0))</f>
+        <v/>
+      </c>
+      <c r="W19" s="27" t="str">
         <f aca="false">IF($B19="","",IF($D19=0,0,$V19/$D19))</f>
         <v/>
       </c>
-      <c r="X19" s="26" t="str">
+      <c r="X19" s="27" t="str">
         <f aca="false">IF($B19="","",IF(($E19+$F19)=0,0,$V19/($E19+$F19)))</f>
         <v/>
       </c>
@@ -2653,55 +2777,55 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
-      <c r="L20" s="24" t="str">
+      <c r="L20" s="25" t="str">
         <f aca="false">IF($B20="","",IFERROR(IF($C20="Premium",INDEX(ComisionPremium,MATCH($B20,CatList,0)),INDEX(ComisionClasica,MATCH($B20,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M20" s="25" t="str">
+      <c r="M20" s="26" t="str">
         <f aca="false">IF($B20="","",$D20*$L20)</f>
         <v/>
       </c>
-      <c r="N20" s="25" t="str">
+      <c r="N20" s="26" t="str">
         <f aca="false">IF($B20="","",IFERROR(IF($I20="No",0,IF($D20&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D20,TramoPrecioDesde,1))*IF($H20="Full",1-INDEX(DescuentoFull,MATCH($J20,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G20,TramoPesoDesde,1))*IF($H20="Full",1-INDEX(DescuentoFull,MATCH($J20,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O20" s="25" t="str">
+      <c r="O20" s="26" t="str">
         <f aca="false">IF($B20="","",IFERROR($D20*INDEX(CargoCuotas,MATCH($K20,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P20" s="25" t="str">
+      <c r="P20" s="26" t="str">
         <f aca="false">IF($B20="","",M20+N20+O20)</f>
         <v/>
       </c>
-      <c r="Q20" s="25" t="str">
+      <c r="Q20" s="26" t="str">
         <f aca="false">IF($B20="","",P20*IVAParam)</f>
         <v/>
       </c>
-      <c r="R20" s="25" t="str">
+      <c r="R20" s="26" t="str">
         <f aca="false">IF($B20="","",IF($H20="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S20" s="25" t="str">
+      <c r="S20" s="26" t="str">
         <f aca="false">IF($B20="","",P20+Q20+R20)</f>
         <v/>
       </c>
-      <c r="T20" s="25" t="str">
+      <c r="T20" s="26" t="str">
         <f aca="false">IF($B20="","",$D20*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U20" s="25" t="str">
+      <c r="U20" s="26" t="str">
         <f aca="false">IF($B20="","",$D20-$S20)</f>
         <v/>
       </c>
-      <c r="V20" s="25" t="str">
-        <f aca="false">IF($B20="","",$U20-$E20-$F20)</f>
-        <v/>
-      </c>
-      <c r="W20" s="26" t="str">
+      <c r="V20" s="26" t="str">
+        <f aca="false">IF($B20="","",$U20-$E20-$F20+IF(CondicionFiscal="Responsable Inscripto",$Q20,0))</f>
+        <v/>
+      </c>
+      <c r="W20" s="27" t="str">
         <f aca="false">IF($B20="","",IF($D20=0,0,$V20/$D20))</f>
         <v/>
       </c>
-      <c r="X20" s="26" t="str">
+      <c r="X20" s="27" t="str">
         <f aca="false">IF($B20="","",IF(($E20+$F20)=0,0,$V20/($E20+$F20)))</f>
         <v/>
       </c>
@@ -2718,55 +2842,55 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
-      <c r="L21" s="24" t="str">
+      <c r="L21" s="25" t="str">
         <f aca="false">IF($B21="","",IFERROR(IF($C21="Premium",INDEX(ComisionPremium,MATCH($B21,CatList,0)),INDEX(ComisionClasica,MATCH($B21,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M21" s="25" t="str">
+      <c r="M21" s="26" t="str">
         <f aca="false">IF($B21="","",$D21*$L21)</f>
         <v/>
       </c>
-      <c r="N21" s="25" t="str">
+      <c r="N21" s="26" t="str">
         <f aca="false">IF($B21="","",IFERROR(IF($I21="No",0,IF($D21&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D21,TramoPrecioDesde,1))*IF($H21="Full",1-INDEX(DescuentoFull,MATCH($J21,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G21,TramoPesoDesde,1))*IF($H21="Full",1-INDEX(DescuentoFull,MATCH($J21,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O21" s="25" t="str">
+      <c r="O21" s="26" t="str">
         <f aca="false">IF($B21="","",IFERROR($D21*INDEX(CargoCuotas,MATCH($K21,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P21" s="25" t="str">
+      <c r="P21" s="26" t="str">
         <f aca="false">IF($B21="","",M21+N21+O21)</f>
         <v/>
       </c>
-      <c r="Q21" s="25" t="str">
+      <c r="Q21" s="26" t="str">
         <f aca="false">IF($B21="","",P21*IVAParam)</f>
         <v/>
       </c>
-      <c r="R21" s="25" t="str">
+      <c r="R21" s="26" t="str">
         <f aca="false">IF($B21="","",IF($H21="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S21" s="25" t="str">
+      <c r="S21" s="26" t="str">
         <f aca="false">IF($B21="","",P21+Q21+R21)</f>
         <v/>
       </c>
-      <c r="T21" s="25" t="str">
+      <c r="T21" s="26" t="str">
         <f aca="false">IF($B21="","",$D21*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U21" s="25" t="str">
+      <c r="U21" s="26" t="str">
         <f aca="false">IF($B21="","",$D21-$S21)</f>
         <v/>
       </c>
-      <c r="V21" s="25" t="str">
-        <f aca="false">IF($B21="","",$U21-$E21-$F21)</f>
-        <v/>
-      </c>
-      <c r="W21" s="26" t="str">
+      <c r="V21" s="26" t="str">
+        <f aca="false">IF($B21="","",$U21-$E21-$F21+IF(CondicionFiscal="Responsable Inscripto",$Q21,0))</f>
+        <v/>
+      </c>
+      <c r="W21" s="27" t="str">
         <f aca="false">IF($B21="","",IF($D21=0,0,$V21/$D21))</f>
         <v/>
       </c>
-      <c r="X21" s="26" t="str">
+      <c r="X21" s="27" t="str">
         <f aca="false">IF($B21="","",IF(($E21+$F21)=0,0,$V21/($E21+$F21)))</f>
         <v/>
       </c>
@@ -2783,55 +2907,55 @@
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
-      <c r="L22" s="24" t="str">
+      <c r="L22" s="25" t="str">
         <f aca="false">IF($B22="","",IFERROR(IF($C22="Premium",INDEX(ComisionPremium,MATCH($B22,CatList,0)),INDEX(ComisionClasica,MATCH($B22,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M22" s="25" t="str">
+      <c r="M22" s="26" t="str">
         <f aca="false">IF($B22="","",$D22*$L22)</f>
         <v/>
       </c>
-      <c r="N22" s="25" t="str">
+      <c r="N22" s="26" t="str">
         <f aca="false">IF($B22="","",IFERROR(IF($I22="No",0,IF($D22&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D22,TramoPrecioDesde,1))*IF($H22="Full",1-INDEX(DescuentoFull,MATCH($J22,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G22,TramoPesoDesde,1))*IF($H22="Full",1-INDEX(DescuentoFull,MATCH($J22,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O22" s="25" t="str">
+      <c r="O22" s="26" t="str">
         <f aca="false">IF($B22="","",IFERROR($D22*INDEX(CargoCuotas,MATCH($K22,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P22" s="25" t="str">
+      <c r="P22" s="26" t="str">
         <f aca="false">IF($B22="","",M22+N22+O22)</f>
         <v/>
       </c>
-      <c r="Q22" s="25" t="str">
+      <c r="Q22" s="26" t="str">
         <f aca="false">IF($B22="","",P22*IVAParam)</f>
         <v/>
       </c>
-      <c r="R22" s="25" t="str">
+      <c r="R22" s="26" t="str">
         <f aca="false">IF($B22="","",IF($H22="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S22" s="25" t="str">
+      <c r="S22" s="26" t="str">
         <f aca="false">IF($B22="","",P22+Q22+R22)</f>
         <v/>
       </c>
-      <c r="T22" s="25" t="str">
+      <c r="T22" s="26" t="str">
         <f aca="false">IF($B22="","",$D22*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U22" s="25" t="str">
+      <c r="U22" s="26" t="str">
         <f aca="false">IF($B22="","",$D22-$S22)</f>
         <v/>
       </c>
-      <c r="V22" s="25" t="str">
-        <f aca="false">IF($B22="","",$U22-$E22-$F22)</f>
-        <v/>
-      </c>
-      <c r="W22" s="26" t="str">
+      <c r="V22" s="26" t="str">
+        <f aca="false">IF($B22="","",$U22-$E22-$F22+IF(CondicionFiscal="Responsable Inscripto",$Q22,0))</f>
+        <v/>
+      </c>
+      <c r="W22" s="27" t="str">
         <f aca="false">IF($B22="","",IF($D22=0,0,$V22/$D22))</f>
         <v/>
       </c>
-      <c r="X22" s="26" t="str">
+      <c r="X22" s="27" t="str">
         <f aca="false">IF($B22="","",IF(($E22+$F22)=0,0,$V22/($E22+$F22)))</f>
         <v/>
       </c>
@@ -2848,55 +2972,55 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
-      <c r="L23" s="24" t="str">
+      <c r="L23" s="25" t="str">
         <f aca="false">IF($B23="","",IFERROR(IF($C23="Premium",INDEX(ComisionPremium,MATCH($B23,CatList,0)),INDEX(ComisionClasica,MATCH($B23,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M23" s="25" t="str">
+      <c r="M23" s="26" t="str">
         <f aca="false">IF($B23="","",$D23*$L23)</f>
         <v/>
       </c>
-      <c r="N23" s="25" t="str">
+      <c r="N23" s="26" t="str">
         <f aca="false">IF($B23="","",IFERROR(IF($I23="No",0,IF($D23&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D23,TramoPrecioDesde,1))*IF($H23="Full",1-INDEX(DescuentoFull,MATCH($J23,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G23,TramoPesoDesde,1))*IF($H23="Full",1-INDEX(DescuentoFull,MATCH($J23,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O23" s="25" t="str">
+      <c r="O23" s="26" t="str">
         <f aca="false">IF($B23="","",IFERROR($D23*INDEX(CargoCuotas,MATCH($K23,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P23" s="25" t="str">
+      <c r="P23" s="26" t="str">
         <f aca="false">IF($B23="","",M23+N23+O23)</f>
         <v/>
       </c>
-      <c r="Q23" s="25" t="str">
+      <c r="Q23" s="26" t="str">
         <f aca="false">IF($B23="","",P23*IVAParam)</f>
         <v/>
       </c>
-      <c r="R23" s="25" t="str">
+      <c r="R23" s="26" t="str">
         <f aca="false">IF($B23="","",IF($H23="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S23" s="25" t="str">
+      <c r="S23" s="26" t="str">
         <f aca="false">IF($B23="","",P23+Q23+R23)</f>
         <v/>
       </c>
-      <c r="T23" s="25" t="str">
+      <c r="T23" s="26" t="str">
         <f aca="false">IF($B23="","",$D23*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U23" s="25" t="str">
+      <c r="U23" s="26" t="str">
         <f aca="false">IF($B23="","",$D23-$S23)</f>
         <v/>
       </c>
-      <c r="V23" s="25" t="str">
-        <f aca="false">IF($B23="","",$U23-$E23-$F23)</f>
-        <v/>
-      </c>
-      <c r="W23" s="26" t="str">
+      <c r="V23" s="26" t="str">
+        <f aca="false">IF($B23="","",$U23-$E23-$F23+IF(CondicionFiscal="Responsable Inscripto",$Q23,0))</f>
+        <v/>
+      </c>
+      <c r="W23" s="27" t="str">
         <f aca="false">IF($B23="","",IF($D23=0,0,$V23/$D23))</f>
         <v/>
       </c>
-      <c r="X23" s="26" t="str">
+      <c r="X23" s="27" t="str">
         <f aca="false">IF($B23="","",IF(($E23+$F23)=0,0,$V23/($E23+$F23)))</f>
         <v/>
       </c>
@@ -2913,55 +3037,55 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
-      <c r="L24" s="24" t="str">
+      <c r="L24" s="25" t="str">
         <f aca="false">IF($B24="","",IFERROR(IF($C24="Premium",INDEX(ComisionPremium,MATCH($B24,CatList,0)),INDEX(ComisionClasica,MATCH($B24,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M24" s="25" t="str">
+      <c r="M24" s="26" t="str">
         <f aca="false">IF($B24="","",$D24*$L24)</f>
         <v/>
       </c>
-      <c r="N24" s="25" t="str">
+      <c r="N24" s="26" t="str">
         <f aca="false">IF($B24="","",IFERROR(IF($I24="No",0,IF($D24&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D24,TramoPrecioDesde,1))*IF($H24="Full",1-INDEX(DescuentoFull,MATCH($J24,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G24,TramoPesoDesde,1))*IF($H24="Full",1-INDEX(DescuentoFull,MATCH($J24,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O24" s="25" t="str">
+      <c r="O24" s="26" t="str">
         <f aca="false">IF($B24="","",IFERROR($D24*INDEX(CargoCuotas,MATCH($K24,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P24" s="25" t="str">
+      <c r="P24" s="26" t="str">
         <f aca="false">IF($B24="","",M24+N24+O24)</f>
         <v/>
       </c>
-      <c r="Q24" s="25" t="str">
+      <c r="Q24" s="26" t="str">
         <f aca="false">IF($B24="","",P24*IVAParam)</f>
         <v/>
       </c>
-      <c r="R24" s="25" t="str">
+      <c r="R24" s="26" t="str">
         <f aca="false">IF($B24="","",IF($H24="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S24" s="25" t="str">
+      <c r="S24" s="26" t="str">
         <f aca="false">IF($B24="","",P24+Q24+R24)</f>
         <v/>
       </c>
-      <c r="T24" s="25" t="str">
+      <c r="T24" s="26" t="str">
         <f aca="false">IF($B24="","",$D24*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U24" s="25" t="str">
+      <c r="U24" s="26" t="str">
         <f aca="false">IF($B24="","",$D24-$S24)</f>
         <v/>
       </c>
-      <c r="V24" s="25" t="str">
-        <f aca="false">IF($B24="","",$U24-$E24-$F24)</f>
-        <v/>
-      </c>
-      <c r="W24" s="26" t="str">
+      <c r="V24" s="26" t="str">
+        <f aca="false">IF($B24="","",$U24-$E24-$F24+IF(CondicionFiscal="Responsable Inscripto",$Q24,0))</f>
+        <v/>
+      </c>
+      <c r="W24" s="27" t="str">
         <f aca="false">IF($B24="","",IF($D24=0,0,$V24/$D24))</f>
         <v/>
       </c>
-      <c r="X24" s="26" t="str">
+      <c r="X24" s="27" t="str">
         <f aca="false">IF($B24="","",IF(($E24+$F24)=0,0,$V24/($E24+$F24)))</f>
         <v/>
       </c>
@@ -2978,55 +3102,55 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
-      <c r="L25" s="24" t="str">
+      <c r="L25" s="25" t="str">
         <f aca="false">IF($B25="","",IFERROR(IF($C25="Premium",INDEX(ComisionPremium,MATCH($B25,CatList,0)),INDEX(ComisionClasica,MATCH($B25,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M25" s="25" t="str">
+      <c r="M25" s="26" t="str">
         <f aca="false">IF($B25="","",$D25*$L25)</f>
         <v/>
       </c>
-      <c r="N25" s="25" t="str">
+      <c r="N25" s="26" t="str">
         <f aca="false">IF($B25="","",IFERROR(IF($I25="No",0,IF($D25&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D25,TramoPrecioDesde,1))*IF($H25="Full",1-INDEX(DescuentoFull,MATCH($J25,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G25,TramoPesoDesde,1))*IF($H25="Full",1-INDEX(DescuentoFull,MATCH($J25,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O25" s="25" t="str">
+      <c r="O25" s="26" t="str">
         <f aca="false">IF($B25="","",IFERROR($D25*INDEX(CargoCuotas,MATCH($K25,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P25" s="25" t="str">
+      <c r="P25" s="26" t="str">
         <f aca="false">IF($B25="","",M25+N25+O25)</f>
         <v/>
       </c>
-      <c r="Q25" s="25" t="str">
+      <c r="Q25" s="26" t="str">
         <f aca="false">IF($B25="","",P25*IVAParam)</f>
         <v/>
       </c>
-      <c r="R25" s="25" t="str">
+      <c r="R25" s="26" t="str">
         <f aca="false">IF($B25="","",IF($H25="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S25" s="25" t="str">
+      <c r="S25" s="26" t="str">
         <f aca="false">IF($B25="","",P25+Q25+R25)</f>
         <v/>
       </c>
-      <c r="T25" s="25" t="str">
+      <c r="T25" s="26" t="str">
         <f aca="false">IF($B25="","",$D25*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U25" s="25" t="str">
+      <c r="U25" s="26" t="str">
         <f aca="false">IF($B25="","",$D25-$S25)</f>
         <v/>
       </c>
-      <c r="V25" s="25" t="str">
-        <f aca="false">IF($B25="","",$U25-$E25-$F25)</f>
-        <v/>
-      </c>
-      <c r="W25" s="26" t="str">
+      <c r="V25" s="26" t="str">
+        <f aca="false">IF($B25="","",$U25-$E25-$F25+IF(CondicionFiscal="Responsable Inscripto",$Q25,0))</f>
+        <v/>
+      </c>
+      <c r="W25" s="27" t="str">
         <f aca="false">IF($B25="","",IF($D25=0,0,$V25/$D25))</f>
         <v/>
       </c>
-      <c r="X25" s="26" t="str">
+      <c r="X25" s="27" t="str">
         <f aca="false">IF($B25="","",IF(($E25+$F25)=0,0,$V25/($E25+$F25)))</f>
         <v/>
       </c>
@@ -3043,55 +3167,55 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
-      <c r="L26" s="24" t="str">
+      <c r="L26" s="25" t="str">
         <f aca="false">IF($B26="","",IFERROR(IF($C26="Premium",INDEX(ComisionPremium,MATCH($B26,CatList,0)),INDEX(ComisionClasica,MATCH($B26,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M26" s="25" t="str">
+      <c r="M26" s="26" t="str">
         <f aca="false">IF($B26="","",$D26*$L26)</f>
         <v/>
       </c>
-      <c r="N26" s="25" t="str">
+      <c r="N26" s="26" t="str">
         <f aca="false">IF($B26="","",IFERROR(IF($I26="No",0,IF($D26&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D26,TramoPrecioDesde,1))*IF($H26="Full",1-INDEX(DescuentoFull,MATCH($J26,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G26,TramoPesoDesde,1))*IF($H26="Full",1-INDEX(DescuentoFull,MATCH($J26,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O26" s="25" t="str">
+      <c r="O26" s="26" t="str">
         <f aca="false">IF($B26="","",IFERROR($D26*INDEX(CargoCuotas,MATCH($K26,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P26" s="25" t="str">
+      <c r="P26" s="26" t="str">
         <f aca="false">IF($B26="","",M26+N26+O26)</f>
         <v/>
       </c>
-      <c r="Q26" s="25" t="str">
+      <c r="Q26" s="26" t="str">
         <f aca="false">IF($B26="","",P26*IVAParam)</f>
         <v/>
       </c>
-      <c r="R26" s="25" t="str">
+      <c r="R26" s="26" t="str">
         <f aca="false">IF($B26="","",IF($H26="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S26" s="25" t="str">
+      <c r="S26" s="26" t="str">
         <f aca="false">IF($B26="","",P26+Q26+R26)</f>
         <v/>
       </c>
-      <c r="T26" s="25" t="str">
+      <c r="T26" s="26" t="str">
         <f aca="false">IF($B26="","",$D26*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U26" s="25" t="str">
+      <c r="U26" s="26" t="str">
         <f aca="false">IF($B26="","",$D26-$S26)</f>
         <v/>
       </c>
-      <c r="V26" s="25" t="str">
-        <f aca="false">IF($B26="","",$U26-$E26-$F26)</f>
-        <v/>
-      </c>
-      <c r="W26" s="26" t="str">
+      <c r="V26" s="26" t="str">
+        <f aca="false">IF($B26="","",$U26-$E26-$F26+IF(CondicionFiscal="Responsable Inscripto",$Q26,0))</f>
+        <v/>
+      </c>
+      <c r="W26" s="27" t="str">
         <f aca="false">IF($B26="","",IF($D26=0,0,$V26/$D26))</f>
         <v/>
       </c>
-      <c r="X26" s="26" t="str">
+      <c r="X26" s="27" t="str">
         <f aca="false">IF($B26="","",IF(($E26+$F26)=0,0,$V26/($E26+$F26)))</f>
         <v/>
       </c>
@@ -3108,55 +3232,55 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
-      <c r="L27" s="24" t="str">
+      <c r="L27" s="25" t="str">
         <f aca="false">IF($B27="","",IFERROR(IF($C27="Premium",INDEX(ComisionPremium,MATCH($B27,CatList,0)),INDEX(ComisionClasica,MATCH($B27,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M27" s="25" t="str">
+      <c r="M27" s="26" t="str">
         <f aca="false">IF($B27="","",$D27*$L27)</f>
         <v/>
       </c>
-      <c r="N27" s="25" t="str">
+      <c r="N27" s="26" t="str">
         <f aca="false">IF($B27="","",IFERROR(IF($I27="No",0,IF($D27&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D27,TramoPrecioDesde,1))*IF($H27="Full",1-INDEX(DescuentoFull,MATCH($J27,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G27,TramoPesoDesde,1))*IF($H27="Full",1-INDEX(DescuentoFull,MATCH($J27,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O27" s="25" t="str">
+      <c r="O27" s="26" t="str">
         <f aca="false">IF($B27="","",IFERROR($D27*INDEX(CargoCuotas,MATCH($K27,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P27" s="25" t="str">
+      <c r="P27" s="26" t="str">
         <f aca="false">IF($B27="","",M27+N27+O27)</f>
         <v/>
       </c>
-      <c r="Q27" s="25" t="str">
+      <c r="Q27" s="26" t="str">
         <f aca="false">IF($B27="","",P27*IVAParam)</f>
         <v/>
       </c>
-      <c r="R27" s="25" t="str">
+      <c r="R27" s="26" t="str">
         <f aca="false">IF($B27="","",IF($H27="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S27" s="25" t="str">
+      <c r="S27" s="26" t="str">
         <f aca="false">IF($B27="","",P27+Q27+R27)</f>
         <v/>
       </c>
-      <c r="T27" s="25" t="str">
+      <c r="T27" s="26" t="str">
         <f aca="false">IF($B27="","",$D27*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U27" s="25" t="str">
+      <c r="U27" s="26" t="str">
         <f aca="false">IF($B27="","",$D27-$S27)</f>
         <v/>
       </c>
-      <c r="V27" s="25" t="str">
-        <f aca="false">IF($B27="","",$U27-$E27-$F27)</f>
-        <v/>
-      </c>
-      <c r="W27" s="26" t="str">
+      <c r="V27" s="26" t="str">
+        <f aca="false">IF($B27="","",$U27-$E27-$F27+IF(CondicionFiscal="Responsable Inscripto",$Q27,0))</f>
+        <v/>
+      </c>
+      <c r="W27" s="27" t="str">
         <f aca="false">IF($B27="","",IF($D27=0,0,$V27/$D27))</f>
         <v/>
       </c>
-      <c r="X27" s="26" t="str">
+      <c r="X27" s="27" t="str">
         <f aca="false">IF($B27="","",IF(($E27+$F27)=0,0,$V27/($E27+$F27)))</f>
         <v/>
       </c>
@@ -3173,55 +3297,55 @@
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
-      <c r="L28" s="24" t="str">
+      <c r="L28" s="25" t="str">
         <f aca="false">IF($B28="","",IFERROR(IF($C28="Premium",INDEX(ComisionPremium,MATCH($B28,CatList,0)),INDEX(ComisionClasica,MATCH($B28,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M28" s="25" t="str">
+      <c r="M28" s="26" t="str">
         <f aca="false">IF($B28="","",$D28*$L28)</f>
         <v/>
       </c>
-      <c r="N28" s="25" t="str">
+      <c r="N28" s="26" t="str">
         <f aca="false">IF($B28="","",IFERROR(IF($I28="No",0,IF($D28&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D28,TramoPrecioDesde,1))*IF($H28="Full",1-INDEX(DescuentoFull,MATCH($J28,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G28,TramoPesoDesde,1))*IF($H28="Full",1-INDEX(DescuentoFull,MATCH($J28,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O28" s="25" t="str">
+      <c r="O28" s="26" t="str">
         <f aca="false">IF($B28="","",IFERROR($D28*INDEX(CargoCuotas,MATCH($K28,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P28" s="25" t="str">
+      <c r="P28" s="26" t="str">
         <f aca="false">IF($B28="","",M28+N28+O28)</f>
         <v/>
       </c>
-      <c r="Q28" s="25" t="str">
+      <c r="Q28" s="26" t="str">
         <f aca="false">IF($B28="","",P28*IVAParam)</f>
         <v/>
       </c>
-      <c r="R28" s="25" t="str">
+      <c r="R28" s="26" t="str">
         <f aca="false">IF($B28="","",IF($H28="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S28" s="25" t="str">
+      <c r="S28" s="26" t="str">
         <f aca="false">IF($B28="","",P28+Q28+R28)</f>
         <v/>
       </c>
-      <c r="T28" s="25" t="str">
+      <c r="T28" s="26" t="str">
         <f aca="false">IF($B28="","",$D28*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U28" s="25" t="str">
+      <c r="U28" s="26" t="str">
         <f aca="false">IF($B28="","",$D28-$S28)</f>
         <v/>
       </c>
-      <c r="V28" s="25" t="str">
-        <f aca="false">IF($B28="","",$U28-$E28-$F28)</f>
-        <v/>
-      </c>
-      <c r="W28" s="26" t="str">
+      <c r="V28" s="26" t="str">
+        <f aca="false">IF($B28="","",$U28-$E28-$F28+IF(CondicionFiscal="Responsable Inscripto",$Q28,0))</f>
+        <v/>
+      </c>
+      <c r="W28" s="27" t="str">
         <f aca="false">IF($B28="","",IF($D28=0,0,$V28/$D28))</f>
         <v/>
       </c>
-      <c r="X28" s="26" t="str">
+      <c r="X28" s="27" t="str">
         <f aca="false">IF($B28="","",IF(($E28+$F28)=0,0,$V28/($E28+$F28)))</f>
         <v/>
       </c>
@@ -3238,55 +3362,55 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
-      <c r="L29" s="24" t="str">
+      <c r="L29" s="25" t="str">
         <f aca="false">IF($B29="","",IFERROR(IF($C29="Premium",INDEX(ComisionPremium,MATCH($B29,CatList,0)),INDEX(ComisionClasica,MATCH($B29,CatList,0))),0))</f>
         <v/>
       </c>
-      <c r="M29" s="25" t="str">
+      <c r="M29" s="26" t="str">
         <f aca="false">IF($B29="","",$D29*$L29)</f>
         <v/>
       </c>
-      <c r="N29" s="25" t="str">
+      <c r="N29" s="26" t="str">
         <f aca="false">IF($B29="","",IFERROR(IF($I29="No",0,IF($D29&lt;UmbralEnvioGratis,INDEX(CostoFijoTramo,MATCH($D29,TramoPrecioDesde,1))*IF($H29="Full",1-INDEX(DescuentoFull,MATCH($J29,ReputacionList,0)),1),INDEX(CostoEnvioPeso,MATCH($G29,TramoPesoDesde,1))*IF($H29="Full",1-INDEX(DescuentoFull,MATCH($J29,ReputacionList,0)),1))),0))</f>
         <v/>
       </c>
-      <c r="O29" s="25" t="str">
+      <c r="O29" s="26" t="str">
         <f aca="false">IF($B29="","",IFERROR($D29*INDEX(CargoCuotas,MATCH($K29,CuotasList,0)),0))</f>
         <v/>
       </c>
-      <c r="P29" s="25" t="str">
+      <c r="P29" s="26" t="str">
         <f aca="false">IF($B29="","",M29+N29+O29)</f>
         <v/>
       </c>
-      <c r="Q29" s="25" t="str">
+      <c r="Q29" s="26" t="str">
         <f aca="false">IF($B29="","",P29*IVAParam)</f>
         <v/>
       </c>
-      <c r="R29" s="25" t="str">
+      <c r="R29" s="26" t="str">
         <f aca="false">IF($B29="","",IF($H29="Full",AlmacenFull,0))</f>
         <v/>
       </c>
-      <c r="S29" s="25" t="str">
+      <c r="S29" s="26" t="str">
         <f aca="false">IF($B29="","",P29+Q29+R29)</f>
         <v/>
       </c>
-      <c r="T29" s="25" t="str">
+      <c r="T29" s="26" t="str">
         <f aca="false">IF($B29="","",$D29*IIBBParam)</f>
         <v/>
       </c>
-      <c r="U29" s="25" t="str">
+      <c r="U29" s="26" t="str">
         <f aca="false">IF($B29="","",$D29-$S29)</f>
         <v/>
       </c>
-      <c r="V29" s="25" t="str">
-        <f aca="false">IF($B29="","",$U29-$E29-$F29)</f>
-        <v/>
-      </c>
-      <c r="W29" s="26" t="str">
+      <c r="V29" s="26" t="str">
+        <f aca="false">IF($B29="","",$U29-$E29-$F29+IF(CondicionFiscal="Responsable Inscripto",$Q29,0))</f>
+        <v/>
+      </c>
+      <c r="W29" s="27" t="str">
         <f aca="false">IF($B29="","",IF($D29=0,0,$V29/$D29))</f>
         <v/>
       </c>
-      <c r="X29" s="26" t="str">
+      <c r="X29" s="27" t="str">
         <f aca="false">IF($B29="","",IF(($E29+$F29)=0,0,$V29/($E29+$F29)))</f>
         <v/>
       </c>
@@ -3350,180 +3474,387 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="D4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="28"/>
+      <c r="G4" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" s="28"/>
+    </row>
+    <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="29" t="n">
+        <f aca="false">COUNT(Calculadora!$D$6:$D$29)</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="D5" s="30" t="n">
+        <f aca="false">IFERROR(AVERAGE(Calculadora!$D$6:$D$29),0)</f>
+        <v>20750</v>
+      </c>
+      <c r="E5" s="30"/>
+      <c r="G5" s="30" t="n">
+        <f aca="false">SUM(Calculadora!$V$6:$V$29)</f>
+        <v>19548.5</v>
+      </c>
+      <c r="H5" s="30"/>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="28"/>
+      <c r="D7" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="28"/>
+      <c r="G7" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="28"/>
+    </row>
+    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="31" t="n">
+        <f aca="false">IFERROR(AVERAGE(Calculadora!$W$6:$W$29),0)</f>
+        <v>0.233397916666667</v>
+      </c>
+      <c r="B8" s="31"/>
+      <c r="D8" s="31" t="n">
+        <f aca="false">IFERROR(AVERAGE(Calculadora!$X$6:$X$29),0)</f>
+        <v>0.457359585628114</v>
+      </c>
+      <c r="E8" s="31"/>
+      <c r="G8" s="32" t="n">
+        <f aca="false">COUNTIFS(Calculadora!$X$6:$X$29,"&lt;0")</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="32"/>
+    </row>
+    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="33"/>
+      <c r="D11" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="33"/>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="34" t="str">
+        <f aca="false">IFERROR(INDEX(Calculadora!$A$6:$A$29,MATCH(MAX(Calculadora!$X$6:$X$29),Calculadora!$X$6:$X$29,0)),"—")</f>
+        <v>EJEMPLO 4 — Producto económico (envío a cargo del comprador, &lt; $33.000)</v>
+      </c>
+      <c r="B12" s="34"/>
+      <c r="D12" s="34" t="str">
+        <f aca="false">IFERROR(INDEX(Calculadora!$A$6:$A$29,MATCH(MIN(Calculadora!$X$6:$X$29),Calculadora!$X$6:$X$29,0)),"—")</f>
+        <v>EJEMPLO 2 — Auricular Bluetooth (Full, envío gratis, &lt; $33.000)</v>
+      </c>
+      <c r="E12" s="34"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="35" t="n">
+        <f aca="false">IFERROR(MAX(Calculadora!$X$6:$X$29),0)</f>
+        <v>0.632487804878049</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="D13" s="35" t="n">
+        <f aca="false">IFERROR(MIN(Calculadora!$X$6:$X$29),0)</f>
+        <v>0.241629032258064</v>
+      </c>
+      <c r="E13" s="35"/>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="A15:H15"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27" t="s">
-        <v>80</v>
+      <c r="A1" s="36" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
-        <v>81</v>
+      <c r="A3" s="37" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
-        <v>82</v>
+      <c r="A4" s="38" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>86</v>
+      <c r="A5" s="38" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="38" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="38" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="37" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>87</v>
+      <c r="A10" s="38" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>88</v>
+      <c r="A11" s="38" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
-        <v>91</v>
+      <c r="A12" s="38" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="38" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="30" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="30" t="s">
-        <v>94</v>
+      <c r="A16" s="38" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="37" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
-        <v>95</v>
+      <c r="A19" s="39" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="s">
-        <v>96</v>
+      <c r="A20" s="39" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="s">
-        <v>97</v>
+      <c r="A21" s="39" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="s">
-        <v>98</v>
+      <c r="A22" s="39" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30" t="s">
-        <v>99</v>
+      <c r="A23" s="39" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="30" t="s">
-        <v>100</v>
+      <c r="A24" s="39" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="30" t="s">
-        <v>101</v>
+      <c r="A25" s="39" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="30" t="s">
-        <v>102</v>
+      <c r="A26" s="39" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="30" t="s">
-        <v>103</v>
+      <c r="A27" s="39" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="30" t="s">
-        <v>104</v>
+      <c r="A28" s="39" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30" t="s">
-        <v>105</v>
+      <c r="A29" s="39" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="30" t="s">
-        <v>106</v>
+      <c r="A30" s="39" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="s">
-        <v>107</v>
+      <c r="A31" s="39" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="30" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29" t="s">
-        <v>109</v>
+      <c r="A32" s="39" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="39" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="39" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="38" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A17" r:id="rId1" display="Costos de ofrecer envío gratis — Ayuda oficial Mercado Libre"/>
-    <hyperlink ref="A18" r:id="rId2" display="Costo por unidad vendida (Full, correo, colecta, puntos de despacho) — Ayuda oficial Mercado Libre"/>
-    <hyperlink ref="A19" r:id="rId3" display="Costos por vender — Mercado Libre Developers"/>
-    <hyperlink ref="A20" r:id="rId4" display="Cómo revisar tus costos diarios por almacenar stock en Full — Mercado Libre Vendedores"/>
-    <hyperlink ref="A21" r:id="rId5" display="Vender con Full — Mercado Envíos"/>
-    <hyperlink ref="A22" r:id="rId6" display="Comisiones MercadoLibre 2026: Tabla por Categoría — SpomBridge"/>
-    <hyperlink ref="A23" r:id="rId7" display="Comisiones de Mercado Libre 2026: tabla por categoría y país — Jaguar Sheet"/>
-    <hyperlink ref="A24" r:id="rId8" display="Comisiones Mercado Libre 2026: Tabla por Categoría — DigitalSellers"/>
-    <hyperlink ref="A25" r:id="rId9" display="¿Cuánto cobra Mercado Libre Argentina por vender? — WooSync"/>
-    <hyperlink ref="A26" r:id="rId10" display="¿Cuánto cuesta vender en Mercado Libre en Argentina? — Base"/>
-    <hyperlink ref="A27" r:id="rId11" display="Cambios de costos, tarifas y envíos en Mercado Libre Argentina 2025 — Academia Nubimetrics"/>
-    <hyperlink ref="A28" r:id="rId12" display="Cuánto cobra realmente Mercado Libre en 2026 (comisiones + IVA) — MargenKit"/>
-    <hyperlink ref="A29" r:id="rId13" display="Mercado Libre desde el 12 de marzo: nuevos costos y rentabilidad real — Enretail"/>
-    <hyperlink ref="A30" r:id="rId14" display="Cuotas sin interés en Mercado Libre: cuántas vale la pena ofrecer — Base"/>
-    <hyperlink ref="A31" r:id="rId15" display="Impuestos en Mercado Libre 2026: Guía Definitiva — Contablix"/>
-    <hyperlink ref="A32" r:id="rId16" display="Retenciones y Percepciones en E-commerce Argentina 2026 — Contablix"/>
+    <hyperlink ref="A19" r:id="rId1" display="Costos de ofrecer envío gratis — Ayuda oficial Mercado Libre"/>
+    <hyperlink ref="A20" r:id="rId2" display="Costo por unidad vendida (Full, correo, colecta, puntos de despacho) — Ayuda oficial Mercado Libre"/>
+    <hyperlink ref="A21" r:id="rId3" display="Costos por vender — Mercado Libre Developers"/>
+    <hyperlink ref="A22" r:id="rId4" display="Cómo revisar tus costos diarios por almacenar stock en Full — Mercado Libre Vendedores"/>
+    <hyperlink ref="A23" r:id="rId5" display="Vender con Full — Mercado Envíos"/>
+    <hyperlink ref="A24" r:id="rId6" display="Comisiones MercadoLibre 2026: Tabla por Categoría — SpomBridge"/>
+    <hyperlink ref="A25" r:id="rId7" display="Comisiones de Mercado Libre 2026: tabla por categoría y país — Jaguar Sheet"/>
+    <hyperlink ref="A26" r:id="rId8" display="Comisiones Mercado Libre 2026: Tabla por Categoría — DigitalSellers"/>
+    <hyperlink ref="A27" r:id="rId9" display="¿Cuánto cobra Mercado Libre Argentina por vender? — WooSync"/>
+    <hyperlink ref="A28" r:id="rId10" display="¿Cuánto cuesta vender en Mercado Libre en Argentina? — Base"/>
+    <hyperlink ref="A29" r:id="rId11" display="Cambios de costos, tarifas y envíos en Mercado Libre Argentina 2025 — Academia Nubimetrics"/>
+    <hyperlink ref="A30" r:id="rId12" display="Cuánto cobra realmente Mercado Libre en 2026 (comisiones + IVA) — MargenKit"/>
+    <hyperlink ref="A31" r:id="rId13" display="Mercado Libre desde el 12 de marzo: nuevos costos y rentabilidad real — Enretail"/>
+    <hyperlink ref="A32" r:id="rId14" display="Cuotas sin interés en Mercado Libre: cuántas vale la pena ofrecer — Base"/>
+    <hyperlink ref="A33" r:id="rId15" display="Impuestos en Mercado Libre 2026: Guía Definitiva — Contablix"/>
+    <hyperlink ref="A34" r:id="rId16" display="Retenciones y Percepciones en E-commerce Argentina 2026 — Contablix"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>